<commit_message>
Avances ETFA - api DM
</commit_message>
<xml_diff>
--- a/Descarga Muestras/Historico.xlsx
+++ b/Descarga Muestras/Historico.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,12 +28,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,19 +48,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -77,7 +64,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -440,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A76"/>
+  <dimension ref="A1:A125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -821,14 +808,259 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" t="n">
+        <v>2310996</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>2327007</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2326412</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>2261909</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>2327978</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>2331147</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>2296367</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2348537</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2348538</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>2348546</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2348554</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>2348555</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>2348556</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>2348557</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>2348558</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>2348559</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>2348560</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>2344733</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>2346386</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>2346391</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>2350375</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>2350374</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>2346369</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>2346380</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>2350379</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>2350376</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>2346367</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>2346364</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>2346368</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>2346385</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>2346383</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>2350373</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>2346388</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>2346374</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2346376</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>2346372</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>2350380</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>2350381</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>2346921</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>2346926</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>2329224</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>2329733</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>2329834</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>2337009</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>2328816</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>2328819</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>2328821</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>2328822</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>2328829</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
         <is>
-          <t>2310996</t>
+          <t>2328835</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A76"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:A125"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Inicio de pruebas ETFA
</commit_message>
<xml_diff>
--- a/Descarga Muestras/Historico.xlsx
+++ b/Descarga Muestras/Historico.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A125"/>
+  <dimension ref="A1:A133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1053,14 +1053,54 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
+      <c r="A125" t="n">
+        <v>2328835</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>1973112</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>2128087</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>2131999</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>2132001</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>2190733</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>2204781</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>2204783</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
         <is>
-          <t>2328835</t>
+          <t>2216085</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A125"/>
+  <autoFilter ref="A1:A133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Avance Acred en Excel
</commit_message>
<xml_diff>
--- a/Descarga Muestras/Historico.xlsx
+++ b/Descarga Muestras/Historico.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$157</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A133"/>
+  <dimension ref="A1:A157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1093,14 +1093,134 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr">
+      <c r="A133" t="n">
+        <v>2216085</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>2215966</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>2261330</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>2262799</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>2280874</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>2280985</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>2283556</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>2283557</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>2289008</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>2291744</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>2291748</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>2292069</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>2310332</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>2311312</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>2313088</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>2313903</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>2323709</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>2323711</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>2325011</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>2329195</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>2329929</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>2330390</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>2330516</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>2337760</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
         <is>
-          <t>2216085</t>
+          <t>2337762</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A133"/>
+  <autoFilter ref="A1:A157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correccion tipo numero de muestra por api
</commit_message>
<xml_diff>
--- a/Descarga Muestras/Historico.xlsx
+++ b/Descarga Muestras/Historico.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$249</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$595</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A249"/>
+  <dimension ref="A1:A595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1686,14 +1686,1744 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" t="inlineStr">
+      <c r="A249" t="n">
+        <v>2358440</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>2070031</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>2081616</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>2127108</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>2127112</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>2139778</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>2139784</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>2198501</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>2215969</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>2216097</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>2263148</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>2263149</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>2263150</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>2263151</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>2263152</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>2263153</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>2263309</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>2263310</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>2263311</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>2263312</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>2263313</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>2263319</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>2263321</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>2263322</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>2263323</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>2263324</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>2263325</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>2263496</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>2263497</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>2263498</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>2263499</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>2263501</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>2263502</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>2263505</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>2263506</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>2263507</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>2263509</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>2263511</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>2263512</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>2263918</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>2263919</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>2272620</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>2272626</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>2272648</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>2273251</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>2273407</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>2273408</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>2273409</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>2274615</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>2274616</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>2274617</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>2274618</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>2274619</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>2274620</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>2274621</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>2280873</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>2291830</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>2291832</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>2291833</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>2291835</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>2308287</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>2308288</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>2308289</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>2308604</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>2308756</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>2316470</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>2318268</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>2318323</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>2318330</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>2318333</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>2318342</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>2318993</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>2319001</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>2319037</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>2319262</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>2319263</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>2319358</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>2319521</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>2319651</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>2319660</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>2319769</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>2319808</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>2319955</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>2319958</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>2320003</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>2320054</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>2320059</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>2320060</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>2320423</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>2320486</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>2320487</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>2320488</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>2320489</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>2320490</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>2320491</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>2325981</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>2325987</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>2327004</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>2327946</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>2327947</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>2327948</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>2327949</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>2327994</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>2327996</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>2328085</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>2329209</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>2329210</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>2329211</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>2329212</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>2329213</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>2329214</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>2329215</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>2329223</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>2329260</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>2329267</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>2329309</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>2329310</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>2329311</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>2329322</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>2329328</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>2329329</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>2329426</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>2329430</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>2329436</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>2329509</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>2329511</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>2329512</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>2329513</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>2329514</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>2329542</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>2329543</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>2329586</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>2329590</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>2329597</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>2329636</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>2329685</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>2329729</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>2329775</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>2329829</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="n">
+        <v>2329848</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="n">
+        <v>2329866</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n">
+        <v>2329908</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="n">
+        <v>2330023</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="n">
+        <v>2330038</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n">
+        <v>2330163</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>2330168</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>2330172</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>2330176</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>2330181</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>2330186</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>2330189</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="n">
+        <v>2330206</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="n">
+        <v>2330207</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="n">
+        <v>2330208</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="n">
+        <v>2330209</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="n">
+        <v>2330210</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>2330212</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="n">
+        <v>2330213</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>2330231</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>2330234</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="n">
+        <v>2330269</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="n">
+        <v>2330314</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="n">
+        <v>2330324</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>2330330</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="n">
+        <v>2330340</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="n">
+        <v>2330347</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="n">
+        <v>2330613</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="n">
+        <v>2330617</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>2330621</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>2330625</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="n">
+        <v>2330718</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>2331815</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>2332144</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>2332357</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="n">
+        <v>2332363</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="n">
+        <v>2342063</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="n">
+        <v>2347437</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="n">
+        <v>2349745</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="n">
+        <v>2349747</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>2349945</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>2350656</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>2350658</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>2350760</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>2351535</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>2351965</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>2353041</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="n">
+        <v>2353045</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>2353047</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>2353051</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>2353055</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>2353056</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="n">
+        <v>2357171</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>2357172</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>2357173</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>2357845</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>2357846</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>2359774</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="n">
+        <v>2359775</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="n">
+        <v>2359826</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="n">
+        <v>2359827</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="n">
+        <v>2359828</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>2360840</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>2360911</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="n">
+        <v>2361146</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="n">
+        <v>2361147</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="n">
+        <v>2361148</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="n">
+        <v>2361184</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="n">
+        <v>2361233</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="n">
+        <v>2361992</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="n">
+        <v>2362192</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="n">
+        <v>2362193</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="n">
+        <v>2362310</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>2362328</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>2362330</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>2362395</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>2362396</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>2362397</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>2362398</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>2362399</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>2362400</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>2362412</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>2362413</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>2362414</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>2362415</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>2362416</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>2362417</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>2362437</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>2362444</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>2362452</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>2362453</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>2362454</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>2362456</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>2362464</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>2362465</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>2362470</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>2362472</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>2362478</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>2362483</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>2362518</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>2362953</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>2362974</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>2364581</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>2365285</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>2365998</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>2366186</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>2366322</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>2366323</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>2366324</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>2366325</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>2366326</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>2366327</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>2367596</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>2368217</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>2368293</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>2368416</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>2368417</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>2368424</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>2369035</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>2369036</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>2369037</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>2369038</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>2369039</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>2369317</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>2369318</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="n">
+        <v>2369693</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="n">
+        <v>2370103</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="n">
+        <v>2370104</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>2370738</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="n">
+        <v>2370739</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="n">
+        <v>2370740</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="n">
+        <v>2371006</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="n">
+        <v>2372886</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="n">
+        <v>2373015</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="n">
+        <v>2373016</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="n">
+        <v>2373017</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="n">
+        <v>2373021</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="n">
+        <v>2373022</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="n">
+        <v>2373024</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="n">
+        <v>2373026</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="n">
+        <v>2373027</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="n">
+        <v>2373631</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="n">
+        <v>2373870</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="n">
+        <v>2373872</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="n">
+        <v>2373874</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="n">
+        <v>2373875</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="n">
+        <v>2373876</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="n">
+        <v>2373877</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="n">
+        <v>2373878</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="n">
+        <v>2373879</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="n">
+        <v>2373880</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="n">
+        <v>2373882</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="n">
+        <v>2373884</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="n">
+        <v>2373885</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="n">
+        <v>2373886</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="n">
+        <v>2373887</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="n">
+        <v>2373888</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="n">
+        <v>2373892</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="n">
+        <v>2373894</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="n">
+        <v>2373896</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="n">
+        <v>2373897</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="n">
+        <v>2373899</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="n">
+        <v>2374987</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="n">
+        <v>2375192</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="n">
+        <v>2375193</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="n">
+        <v>2375231</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="n">
+        <v>2375237</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="n">
+        <v>2375327</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="n">
+        <v>2375356</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="n">
+        <v>2375359</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>2376547</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="n">
+        <v>2377108</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>2377109</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>2377110</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="n">
+        <v>2377229</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="n">
+        <v>2377264</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="n">
+        <v>2377372</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="n">
+        <v>2377519</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="n">
+        <v>2378213</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="n">
+        <v>2378633</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="n">
+        <v>2378634</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="n">
+        <v>2378635</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="n">
+        <v>2378636</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="n">
+        <v>2378637</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="n">
+        <v>2378638</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="n">
+        <v>2378639</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="n">
+        <v>2378717</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="n">
+        <v>2378724</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="n">
+        <v>2378727</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="n">
+        <v>2378732</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="n">
+        <v>2378739</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="n">
+        <v>2378745</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="n">
+        <v>2378823</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="n">
+        <v>2378830</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="n">
+        <v>2378831</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="n">
+        <v>2378832</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="n">
+        <v>2378837</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="n">
+        <v>2378838</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="n">
+        <v>2378840</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="n">
+        <v>2378843</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="n">
+        <v>2378855</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="n">
+        <v>2378929</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="n">
+        <v>2378932</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="n">
+        <v>2378933</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="n">
+        <v>2378935</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="n">
+        <v>2378939</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="n">
+        <v>2378942</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
         <is>
-          <t>2358440</t>
+          <t>2378943</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A249"/>
+  <autoFilter ref="A1:A595"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>